<commit_message>
update portfolio & students
</commit_message>
<xml_diff>
--- a/markdown_generator/students.xlsx
+++ b/markdown_generator/students.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiahuanpei/Code/Jiahuan-Pei.github.io/markdown_generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09DD35F0-CEC9-1C4C-A0C3-01849D5CDA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF0BAD3-623F-3C46-B4A5-BDB28C8A3DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="26240" windowHeight="15520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="107">
   <si>
     <t>#</t>
   </si>
@@ -91,9 +91,6 @@
     <t>University of Amsterdam / Centrum Wiskunde &amp; Informatica</t>
   </si>
   <si>
-    <t>From Aligned Models to Trusted Interfaces: Explainable Health Intervention and Transparent Health Information Seeking (Research)</t>
-  </si>
-  <si>
     <t>01/09/2024</t>
   </si>
   <si>
@@ -227,13 +224,130 @@
   </si>
   <si>
     <t>25/10/2025</t>
+  </si>
+  <si>
+    <t>Psycholinguistic Dialogue Generation (Research)</t>
+  </si>
+  <si>
+    <t>Mithat Can Ozgun</t>
+  </si>
+  <si>
+    <t>15/10/2024</t>
+  </si>
+  <si>
+    <t>18/06/2025</t>
+  </si>
+  <si>
+    <t>Xiao Fu</t>
+  </si>
+  <si>
+    <t>09/12/2024</t>
+  </si>
+  <si>
+    <t>15/08/2025</t>
+  </si>
+  <si>
+    <t>Dingming Liu</t>
+  </si>
+  <si>
+    <t>Trustworthy AI Psychotherapy: Multi-Agent LLM Workflow for Counseling and Explainable Mental Disorder Diagnosis (Thesis =&gt; CIKM25)</t>
+  </si>
+  <si>
+    <t>Multi-Agent Simulation of Client-Therapist Dialogues with Large Language Models: An MI-Centered Framework (Thesis =&gt; ACL26)</t>
+  </si>
+  <si>
+    <t>Evaluating Mathematical Reasoning Abilities of Large Language Models within Scientific Literature (Thesis =&gt; ACL26)</t>
+  </si>
+  <si>
+    <t>21/10/2024</t>
+  </si>
+  <si>
+    <t>10/07/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yas Lotfi </t>
+  </si>
+  <si>
+    <t>Explainable Conversational Agent for Mental Health Chatbots Using LLMs</t>
+  </si>
+  <si>
+    <t>17/01/2025</t>
+  </si>
+  <si>
+    <t>25/06/2025</t>
+  </si>
+  <si>
+    <t>Design, Implementation and Evaluation of Vision and Language Agents for LEGO Assembly in Augmented Reality</t>
+  </si>
+  <si>
+    <t>Mkita Yurchyk</t>
+  </si>
+  <si>
+    <t>08/04/2025</t>
+  </si>
+  <si>
+    <t>27/11/2025</t>
+  </si>
+  <si>
+    <t>Thomas Glatz</t>
+  </si>
+  <si>
+    <t>Digital Employee with LLMs</t>
+  </si>
+  <si>
+    <t>07-10-2025</t>
+  </si>
+  <si>
+    <t>Hristina Chalokova</t>
+  </si>
+  <si>
+    <t>19-11-2025</t>
+  </si>
+  <si>
+    <t>Soften Resistance in LLM Mental Health Agents</t>
+  </si>
+  <si>
+    <t>Jiaqi Shi</t>
+  </si>
+  <si>
+    <t>Real-Time Cognitive Load Classification for Adaptive Online Learning Systems</t>
+  </si>
+  <si>
+    <t>17/12/2025</t>
+  </si>
+  <si>
+    <t>Chi Zhang</t>
+  </si>
+  <si>
+    <t>Pre-play – visual communication for everyday autistic life</t>
+  </si>
+  <si>
+    <t>14/01/2026</t>
+  </si>
+  <si>
+    <t>Marouan Hmidach</t>
+  </si>
+  <si>
+    <t>Learning-to-Ask Agent for Structured Report Generation in Special Education</t>
+  </si>
+  <si>
+    <t>17/03/2026</t>
+  </si>
+  <si>
+    <t>Jason Wang</t>
+  </si>
+  <si>
+    <t>Gaze Language Models for Mental Health Support</t>
+  </si>
+  <si>
+    <t>02-12-2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -245,6 +359,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -283,7 +403,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -299,6 +419,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -602,7 +734,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" style="3"/>
@@ -610,8 +742,8 @@
     <col min="3" max="3" width="10.5" style="3" customWidth="1"/>
     <col min="4" max="4" width="46.1640625" style="4" customWidth="1"/>
     <col min="5" max="5" width="65.83203125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="13" style="3" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="13" style="6" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" style="6" customWidth="1"/>
     <col min="8" max="16384" width="8.83203125" style="3"/>
   </cols>
   <sheetData>
@@ -631,10 +763,10 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
     </row>
@@ -654,10 +786,10 @@
       <c r="E2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="6" t="s">
         <v>12</v>
       </c>
     </row>
@@ -677,10 +809,10 @@
       <c r="E3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="6" t="s">
         <v>17</v>
       </c>
     </row>
@@ -700,14 +832,14 @@
       <c r="E4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -721,13 +853,13 @@
         <v>22</v>
       </c>
       <c r="E5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -735,22 +867,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -758,22 +890,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>30</v>
+      <c r="G7" s="6" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -781,22 +913,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E8" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>30</v>
+      <c r="G8" s="6" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -804,22 +936,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -827,22 +959,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -850,22 +982,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E11" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="6" t="s">
         <v>49</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -873,21 +1005,21 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="F12" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="6" t="s">
         <v>12</v>
       </c>
     </row>
@@ -896,22 +1028,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="F13" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="32" x14ac:dyDescent="0.2">
@@ -919,22 +1051,22 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" s="5" t="s">
+      <c r="F14" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" x14ac:dyDescent="0.2">
@@ -942,22 +1074,275 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="F15" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>30</v>
+      <c r="G15" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>